<commit_message>
fix: prevent skipping participants from same department
</commit_message>
<xml_diff>
--- a/data/master_absensi.xlsx
+++ b/data/master_absensi.xlsx
@@ -45,13 +45,13 @@
     <t>Keterlambatan (menit)</t>
   </si>
   <si>
-    <t>ATT-1791535331605-431</t>
-  </si>
-  <si>
-    <t>2026-10-09</t>
-  </si>
-  <si>
-    <t>15:42:11</t>
+    <t>ATT-1792393452708-298</t>
+  </si>
+  <si>
+    <t>2026-10-19</t>
+  </si>
+  <si>
+    <t>14:04:12</t>
   </si>
   <si>
     <t>Siti Rahma</t>
@@ -72,7 +72,7 @@
     <t>20 menit</t>
   </si>
   <si>
-    <t>ATT-1791535331604-516</t>
+    <t>ATT-1792393452705-394</t>
   </si>
   <si>
     <t>Budi Santoso</t>

</xml_diff>

<commit_message>
feat: add Data Karyawan sheet with 14 departments dropdown and individual/division performance monitoring
</commit_message>
<xml_diff>
--- a/data/master_absensi.xlsx
+++ b/data/master_absensi.xlsx
@@ -7,13 +7,14 @@
     <sheet sheetId="1" name="Log Absensi" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Performa Individu" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Rekap Departemen" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="Data Karyawan" state="visible" r:id="rId7"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="41">
   <si>
     <t>No</t>
   </si>
@@ -45,13 +46,13 @@
     <t>Keterlambatan (menit)</t>
   </si>
   <si>
-    <t>ATT-1792393452708-298</t>
-  </si>
-  <si>
-    <t>2026-10-19</t>
-  </si>
-  <si>
-    <t>14:04:12</t>
+    <t>ATT-1792636873584-986</t>
+  </si>
+  <si>
+    <t>2026-10-22</t>
+  </si>
+  <si>
+    <t>09:41:13</t>
   </si>
   <si>
     <t>Siti Rahma</t>
@@ -72,7 +73,7 @@
     <t>20 menit</t>
   </si>
   <si>
-    <t>ATT-1792393452705-394</t>
+    <t>ATT-1792636873583-430</t>
   </si>
   <si>
     <t>Budi Santoso</t>
@@ -118,6 +119,24 @@
   </si>
   <si>
     <t>Total Kehadiran</t>
+  </si>
+  <si>
+    <t>Nama Lengkap Karyawan</t>
+  </si>
+  <si>
+    <t>Departemen / Divisi</t>
+  </si>
+  <si>
+    <t>% On-Time</t>
+  </si>
+  <si>
+    <t>Status Performa</t>
+  </si>
+  <si>
+    <t>⭐ Sangat Baik</t>
+  </si>
+  <si>
+    <t>⚠️ Perlu Ditingkatkan</t>
   </si>
 </sst>
 </file>
@@ -149,7 +168,7 @@
       <b/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -181,6 +200,11 @@
         <fgColor rgb="4338CA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0F172A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -194,7 +218,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -224,6 +248,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -855,4 +882,106 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="3">
+        <v>1</v>
+      </c>
+      <c r="E2" s="3">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3">
+        <v>0</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3">
+        <v>1</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" sqref="C2:C500">
+      <formula1>"EBS,Solution Architect,Could Automation,Research and innovation,Infrastructur Analytic,FAT,Sales,Cyber Cecurity,PMO,BOD,Modern Application,Data Analytics,HCMC,PKL/Magang"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: keep Data Karyawan sheet blank for manual input, link Zoom attendance with department lookup, and add sync feature
</commit_message>
<xml_diff>
--- a/data/master_absensi.xlsx
+++ b/data/master_absensi.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="39">
   <si>
     <t>No</t>
   </si>
@@ -46,13 +46,13 @@
     <t>Keterlambatan (menit)</t>
   </si>
   <si>
-    <t>ATT-1792636873584-986</t>
+    <t>ATT-1792638007211-969</t>
   </si>
   <si>
     <t>2026-10-22</t>
   </si>
   <si>
-    <t>09:41:13</t>
+    <t>10:00:07</t>
   </si>
   <si>
     <t>Siti Rahma</t>
@@ -73,7 +73,7 @@
     <t>20 menit</t>
   </si>
   <si>
-    <t>ATT-1792636873583-430</t>
+    <t>ATT-1792638007210-599</t>
   </si>
   <si>
     <t>Budi Santoso</t>
@@ -131,12 +131,6 @@
   </si>
   <si>
     <t>Status Performa</t>
-  </si>
-  <si>
-    <t>⭐ Sangat Baik</t>
-  </si>
-  <si>
-    <t>⚠️ Perlu Ditingkatkan</t>
   </si>
 </sst>
 </file>
@@ -886,7 +880,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -923,58 +917,6 @@
         <v>38</v>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="3">
-        <v>1</v>
-      </c>
-      <c r="E2" s="3">
-        <v>1</v>
-      </c>
-      <c r="F2" s="3">
-        <v>0</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" s="3">
-        <v>1</v>
-      </c>
-      <c r="E3" s="3">
-        <v>0</v>
-      </c>
-      <c r="F3" s="3">
-        <v>1</v>
-      </c>
-      <c r="G3" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>40</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="C2:C500">

</xml_diff>